<commit_message>
[modify] finish gun init flow.
</commit_message>
<xml_diff>
--- a/DemoDesign/Config/bullet.xlsx
+++ b/DemoDesign/Config/bullet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39DE89C9-AC45-47BB-BCA9-2F3CA3D6B17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C503889-90A1-4575-B4F5-06DE9F228C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>int</t>
   </si>
@@ -158,6 +158,22 @@
   </si>
   <si>
     <t>mass</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bullet/Bullet</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>炮弹预制体路径</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>prefabPath</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>string</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -567,14 +583,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="16.625" defaultRowHeight="28.5" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="20.375" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="16.625" style="7"/>
+    <col min="4" max="4" width="16.625" style="7"/>
+    <col min="5" max="5" width="26" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="16.625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -587,8 +605,11 @@
       <c r="D1" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -601,8 +622,11 @@
       <c r="D2" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="E2" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -615,8 +639,11 @@
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -628,6 +655,9 @@
       </c>
       <c r="D4" s="7" t="s">
         <v>17</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[modify] update monster read config.
</commit_message>
<xml_diff>
--- a/DemoDesign/Config/bullet.xlsx
+++ b/DemoDesign/Config/bullet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C503889-90A1-4575-B4F5-06DE9F228C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A407B9-979D-4777-B285-82FEB160ACD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,10 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
-  <si>
-    <t>int</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>id</t>
   </si>
@@ -174,6 +171,22 @@
   </si>
   <si>
     <t>string</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>移动速度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>moveSpeed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>float</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -583,81 +596,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="16.625" defaultRowHeight="28.5" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="20.375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="16.625" style="7"/>
-    <col min="5" max="5" width="26" style="7" customWidth="1"/>
-    <col min="6" max="16384" width="16.625" style="7"/>
+    <col min="1" max="2" width="20.375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.625" style="7"/>
+    <col min="4" max="5" width="20.375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="26" style="7" customWidth="1"/>
+    <col min="7" max="16384" width="16.625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>18</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -681,22 +707,22 @@
   <sheetData>
     <row r="1" spans="1:1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>